<commit_message>
Introduction TU MV Cas S04
</commit_message>
<xml_diff>
--- a/Manuel Validation/CAS S03/Cas S03.xlsx
+++ b/Manuel Validation/CAS S03/Cas S03.xlsx
@@ -537,7 +537,7 @@
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="0.0000"/>
     <numFmt numFmtId="166" formatCode="0.000"/>
-    <numFmt numFmtId="168" formatCode="0.00000"/>
+    <numFmt numFmtId="167" formatCode="0.00000"/>
   </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
@@ -818,7 +818,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="80">
+  <cellXfs count="81">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -972,7 +972,7 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
@@ -984,7 +984,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="168" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -1001,6 +1001,9 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="0" fillId="13" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="13" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2111,7 +2114,7 @@
         <v>95</v>
       </c>
       <c r="U40" s="62">
-        <f t="shared" ref="U40:U43" si="0">S40*T40/1000</f>
+        <f t="shared" ref="U40:U42" si="0">S40*T40/1000</f>
         <v>29.782499999999999</v>
       </c>
     </row>
@@ -2185,7 +2188,7 @@
       <c r="P43" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="Q43" s="64">
+      <c r="Q43" s="80">
         <f>(Nfs*ABS(zANP-tfs/2)+Nfi*ABS(zANP-(Ht-tfi/2))+Nw*hw/2*(pW^2+(1-pW)^2))/1000</f>
         <v>275.88</v>
       </c>
@@ -2512,8 +2515,8 @@
         <v>135</v>
       </c>
       <c r="N69" s="61">
-        <f>-qQ_1*La^2*LL/18/SQRT(3)/(E*InertieCM4/100)*1000^2</f>
-        <v>-4.4387477937325341</v>
+        <f>-qQ_1*La^2*LL^2/18/SQRT(3)/(E*InertieCM4/100)*1000^2</f>
+        <v>-39.948730143592805</v>
       </c>
       <c r="O69" t="s">
         <v>7</v>
@@ -2670,7 +2673,7 @@
         <v>124</v>
       </c>
       <c r="E90" s="5">
-        <v>4189</v>
+        <v>279</v>
       </c>
       <c r="F90" t="s">
         <v>23</v>
@@ -2682,7 +2685,7 @@
       </c>
       <c r="E91" s="59">
         <f>SQRT(MRd*GammaM0/Mcr)</f>
-        <v>0.25662852539759506</v>
+        <v>0.99439288226589551</v>
       </c>
     </row>
     <row r="92" spans="3:6" x14ac:dyDescent="0.25">
@@ -2699,7 +2702,7 @@
       </c>
       <c r="E93" s="60">
         <f>0.5*(1+AlphaLT*(LambdaLT-0.2)+LambdaLT^2)</f>
-        <v>0.5544479396749582</v>
+        <v>1.2962778974115778</v>
       </c>
     </row>
     <row r="94" spans="3:6" x14ac:dyDescent="0.25">
@@ -2708,7 +2711,7 @@
       </c>
       <c r="E94" s="69">
         <f>1/(PhiLT+SQRT(PhiLT^2-LambdaLT^2))</f>
-        <v>0.95608720441625272</v>
+        <v>0.46995700637303306</v>
       </c>
     </row>
     <row r="95" spans="3:6" x14ac:dyDescent="0.25">
@@ -2717,7 +2720,7 @@
       </c>
       <c r="E95" s="62">
         <f>KhiLT*MRd*GammaM0/GammaM1</f>
-        <v>263.7653379543558</v>
+        <v>129.65173891819236</v>
       </c>
       <c r="F95" t="s">
         <v>23</v>
@@ -2733,7 +2736,7 @@
       </c>
       <c r="E97" s="75">
         <f>MEd_U1/E95</f>
-        <v>-0.88857391883901837</v>
+        <v>-1.8077273930578432</v>
       </c>
     </row>
     <row r="98" spans="4:5" x14ac:dyDescent="0.25">

</xml_diff>